<commit_message>
Complete Study 002 effect size analysis
</commit_message>
<xml_diff>
--- a/research/study_002_foundation_model_comparison/analysis/statistical_outputs/effect_sizes.xlsx
+++ b/research/study_002_foundation_model_comparison/analysis/statistical_outputs/effect_sizes.xlsx
@@ -1,25 +1,134 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
-  <fileVersion appName="xl" lastEdited="6" lowestEdited="6" rupBuild="14420"/>
-  <workbookPr defaultThemeVersion="164011"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29929"/>
+  <workbookPr/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice Requires="x15">
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\3-6-2023\muawia 03-06-2026\Agentic-AI-research\research\study_002_foundation_model_comparison\analysis\statistical_outputs\"/>
+    </mc:Choice>
+  </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{56A2AE15-5B47-49EE-AC86-CC6FADCB2C3B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="22260" windowHeight="12645"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
-    <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
+    <sheet name="Overview" sheetId="2" r:id="rId1"/>
+    <sheet name="Quality_Effect_Sizes" sheetId="3" r:id="rId2"/>
+    <sheet name="Confidence_Effect_Sizes" sheetId="4" r:id="rId3"/>
+    <sheet name="Combined_Effect_Sizes" sheetId="5" r:id="rId4"/>
+    <sheet name="Interpretation" sheetId="6" r:id="rId5"/>
   </sheets>
-  <calcPr calcId="162913"/>
-  <extLst>
-    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
-      <x15:workbookPr chartTrackingRefBase="1"/>
-    </ext>
-  </extLst>
+  <calcPr calcId="0"/>
 </workbook>
 </file>
 
+<file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="102" uniqueCount="33">
+  <si>
+    <t>Item</t>
+  </si>
+  <si>
+    <t>Value</t>
+  </si>
+  <si>
+    <t>Source File</t>
+  </si>
+  <si>
+    <t>anova_results.xlsx</t>
+  </si>
+  <si>
+    <t>Effect Size Metric</t>
+  </si>
+  <si>
+    <t>Partial Eta Squared</t>
+  </si>
+  <si>
+    <t>Primary Outcome</t>
+  </si>
+  <si>
+    <t>quality_score</t>
+  </si>
+  <si>
+    <t>Secondary Outcome</t>
+  </si>
+  <si>
+    <t>confidence</t>
+  </si>
+  <si>
+    <t>Interpretation Thresholds</t>
+  </si>
+  <si>
+    <t>0.01 = Small, 0.06 = Medium, 0.14 = Large</t>
+  </si>
+  <si>
+    <t>Status</t>
+  </si>
+  <si>
+    <t>Completed</t>
+  </si>
+  <si>
+    <t>Outcome</t>
+  </si>
+  <si>
+    <t>Source</t>
+  </si>
+  <si>
+    <t>Partial_Eta_Squared</t>
+  </si>
+  <si>
+    <t>Interpretation</t>
+  </si>
+  <si>
+    <t>Significant</t>
+  </si>
+  <si>
+    <t>Provider</t>
+  </si>
+  <si>
+    <t>Small</t>
+  </si>
+  <si>
+    <t>Yes</t>
+  </si>
+  <si>
+    <t>Workflow</t>
+  </si>
+  <si>
+    <t>Medium</t>
+  </si>
+  <si>
+    <t>Provider × Workflow</t>
+  </si>
+  <si>
+    <t>No</t>
+  </si>
+  <si>
+    <t>Threshold</t>
+  </si>
+  <si>
+    <t>&lt; 0.01</t>
+  </si>
+  <si>
+    <t>Negligible</t>
+  </si>
+  <si>
+    <t>0.01 to &lt; 0.06</t>
+  </si>
+  <si>
+    <t>0.06 to &lt; 0.14</t>
+  </si>
+  <si>
+    <t>&gt;= 0.14</t>
+  </si>
+  <si>
+    <t>Large</t>
+  </si>
+</sst>
+</file>
+
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <fonts count="1" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
@@ -49,13 +158,101 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="0"/>
+  <dxfs count="28">
+    <dxf>
+      <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+  </dxfs>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
@@ -66,6 +263,73 @@
     </ext>
   </extLst>
 </styleSheet>
+</file>
+
+<file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{F322F92D-BF98-4FEF-A49B-82EB08541FBC}" name="Table1" displayName="Table1" ref="A1:B7" totalsRowShown="0">
+  <autoFilter ref="A1:B7" xr:uid="{F322F92D-BF98-4FEF-A49B-82EB08541FBC}"/>
+  <tableColumns count="2">
+    <tableColumn id="1" xr3:uid="{BB982AA3-0A01-41F0-A187-C28B3F267CF7}" name="Item"/>
+    <tableColumn id="2" xr3:uid="{DB07B041-F414-483E-AF97-F346CAB66900}" name="Value"/>
+  </tableColumns>
+  <tableStyleInfo name="TableStyleMedium9" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
+</table>
+</file>
+
+<file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{5D6EAEEC-A0F6-4E4D-B85F-5386A555644F}" name="Table2" displayName="Table2" ref="A1:F4" totalsRowShown="0" headerRowDxfId="21" dataDxfId="20">
+  <autoFilter ref="A1:F4" xr:uid="{5D6EAEEC-A0F6-4E4D-B85F-5386A555644F}"/>
+  <tableColumns count="6">
+    <tableColumn id="1" xr3:uid="{0453AE8A-13D3-4FD9-9796-E5E74C9B0B65}" name="Outcome" dataDxfId="27"/>
+    <tableColumn id="2" xr3:uid="{D0B8F821-AFE7-4F2C-88F4-4DFB342A281A}" name="Source" dataDxfId="26"/>
+    <tableColumn id="3" xr3:uid="{0132AAAB-D206-43FD-829C-BD3195DA53C3}" name="Partial_Eta_Squared" dataDxfId="25"/>
+    <tableColumn id="4" xr3:uid="{3C9C83DB-D33D-406C-A13E-38DE65C0D7BE}" name="Effect Size Metric" dataDxfId="24"/>
+    <tableColumn id="5" xr3:uid="{CD105EDA-1D76-4499-81A9-59424FCC47B1}" name="Interpretation" dataDxfId="23"/>
+    <tableColumn id="6" xr3:uid="{4E289E2E-CDD9-493C-8930-54BE944DEB81}" name="Significant" dataDxfId="22"/>
+  </tableColumns>
+  <tableStyleInfo name="TableStyleMedium9" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
+</table>
+</file>
+
+<file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="3" xr:uid="{AF901B83-2FB6-4CD0-91D3-7A869DD8D674}" name="Table3" displayName="Table3" ref="A1:F4" totalsRowShown="0" headerRowDxfId="13" dataDxfId="12">
+  <autoFilter ref="A1:F4" xr:uid="{AF901B83-2FB6-4CD0-91D3-7A869DD8D674}"/>
+  <tableColumns count="6">
+    <tableColumn id="1" xr3:uid="{3ED47208-9D9E-4A9B-9BA3-DCE6495DF2C9}" name="Outcome" dataDxfId="19"/>
+    <tableColumn id="2" xr3:uid="{3F2BA2C2-2C94-4C77-A2F6-F4ADC6A89720}" name="Source" dataDxfId="18"/>
+    <tableColumn id="3" xr3:uid="{5CC05EB9-3E64-4A91-81A2-5B4B26C39A25}" name="Partial_Eta_Squared" dataDxfId="17"/>
+    <tableColumn id="4" xr3:uid="{D93E0240-E966-4EBD-ABCA-A0DC15F09370}" name="Effect Size Metric" dataDxfId="16"/>
+    <tableColumn id="5" xr3:uid="{A48CED9E-7A90-4C95-AE95-C360D7862E50}" name="Interpretation" dataDxfId="15"/>
+    <tableColumn id="6" xr3:uid="{5DC3BFED-8225-4503-B69F-B3CB467651B9}" name="Significant" dataDxfId="14"/>
+  </tableColumns>
+  <tableStyleInfo name="TableStyleMedium9" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
+</table>
+</file>
+
+<file path=xl/tables/table4.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="4" xr:uid="{3DDB7BEC-2BB6-41D7-A9D3-AF85D630209F}" name="Table4" displayName="Table4" ref="A1:F7" totalsRowShown="0" headerRowDxfId="5" dataDxfId="4">
+  <autoFilter ref="A1:F7" xr:uid="{3DDB7BEC-2BB6-41D7-A9D3-AF85D630209F}"/>
+  <tableColumns count="6">
+    <tableColumn id="1" xr3:uid="{345BF9C7-CDD3-45E7-A468-EA25D8C00AFD}" name="Outcome" dataDxfId="11"/>
+    <tableColumn id="2" xr3:uid="{30F8E424-C237-46D3-B8F7-E86C55E23E56}" name="Source" dataDxfId="10"/>
+    <tableColumn id="3" xr3:uid="{176334A9-85CA-4396-AAA5-0A484BC60514}" name="Partial_Eta_Squared" dataDxfId="9"/>
+    <tableColumn id="4" xr3:uid="{870EC168-2BA8-4D35-947D-1DD33E290036}" name="Effect Size Metric" dataDxfId="8"/>
+    <tableColumn id="5" xr3:uid="{D5F9086B-1FA3-4EC1-A708-3E0085C6008C}" name="Interpretation" dataDxfId="7"/>
+    <tableColumn id="6" xr3:uid="{43AB5109-3DC6-42E3-8717-4537B565612F}" name="Significant" dataDxfId="6"/>
+  </tableColumns>
+  <tableStyleInfo name="TableStyleMedium9" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
+</table>
+</file>
+
+<file path=xl/tables/table5.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="5" xr:uid="{4FDB893D-56C6-4580-AF35-7D5E66E44DA3}" name="Table5" displayName="Table5" ref="A1:B5" totalsRowShown="0" headerRowDxfId="1" dataDxfId="0">
+  <autoFilter ref="A1:B5" xr:uid="{4FDB893D-56C6-4580-AF35-7D5E66E44DA3}"/>
+  <tableColumns count="2">
+    <tableColumn id="1" xr3:uid="{5D59D4F9-9EEF-4AA4-B748-9208EB35EA61}" name="Threshold" dataDxfId="3"/>
+    <tableColumn id="2" xr3:uid="{77BED6BC-488E-44B3-81CA-D3CCE7677661}" name="Interpretation" dataDxfId="2"/>
+  </tableColumns>
+  <tableStyleInfo name="TableStyleMedium9" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
+</table>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -330,10 +594,492 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
-  <sheetData/>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
+  <dimension ref="A1:B7"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="1" max="1" width="22" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="35.21875" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="2" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A2" t="s">
+        <v>2</v>
+      </c>
+      <c r="B2" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="3" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A3" t="s">
+        <v>4</v>
+      </c>
+      <c r="B3" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="4" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A4" t="s">
+        <v>6</v>
+      </c>
+      <c r="B4" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="5" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A5" t="s">
+        <v>8</v>
+      </c>
+      <c r="B5" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="6" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A6" t="s">
+        <v>10</v>
+      </c>
+      <c r="B6" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="7" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A7" t="s">
+        <v>12</v>
+      </c>
+      <c r="B7" t="s">
+        <v>13</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <tableParts count="1">
+    <tablePart r:id="rId1"/>
+  </tableParts>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
+  <dimension ref="A1:F4"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="1" max="1" width="10.44140625" customWidth="1"/>
+    <col min="3" max="3" width="19.33203125" customWidth="1"/>
+    <col min="4" max="4" width="17.77734375" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="15" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="11.21875" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A1" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>16</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="E1" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="F1" s="1" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="2" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A2" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="B2" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="C2" s="1">
+        <v>2.3830198725143099E-2</v>
+      </c>
+      <c r="D2" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="E2" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="F2" s="1" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="3" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A3" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="B3" s="1" t="s">
+        <v>22</v>
+      </c>
+      <c r="C3" s="1">
+        <v>9.8940003930462081E-2</v>
+      </c>
+      <c r="D3" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="E3" s="1" t="s">
+        <v>23</v>
+      </c>
+      <c r="F3" s="1" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="4" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A4" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="B4" s="1" t="s">
+        <v>24</v>
+      </c>
+      <c r="C4" s="1">
+        <v>6.6832214140167642E-2</v>
+      </c>
+      <c r="D4" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="E4" s="1" t="s">
+        <v>23</v>
+      </c>
+      <c r="F4" s="1" t="s">
+        <v>21</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <tableParts count="1">
+    <tablePart r:id="rId1"/>
+  </tableParts>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0300-000000000000}">
+  <dimension ref="A1:F4"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="1" max="1" width="11" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="18" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="20.44140625" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="17.77734375" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="14.33203125" customWidth="1"/>
+    <col min="6" max="6" width="11.21875" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A1" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>16</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="E1" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="F1" s="1" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="2" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A2" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="B2" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="C2" s="1">
+        <v>8.554868239026639E-2</v>
+      </c>
+      <c r="D2" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="E2" s="1" t="s">
+        <v>23</v>
+      </c>
+      <c r="F2" s="1" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="3" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A3" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="B3" s="1" t="s">
+        <v>22</v>
+      </c>
+      <c r="C3" s="1">
+        <v>2.7019692250728311E-2</v>
+      </c>
+      <c r="D3" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="E3" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="F3" s="1" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="4" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A4" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="B4" s="1" t="s">
+        <v>24</v>
+      </c>
+      <c r="C4" s="1">
+        <v>3.0057600886604991E-2</v>
+      </c>
+      <c r="D4" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="E4" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="F4" s="1" t="s">
+        <v>25</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <tableParts count="1">
+    <tablePart r:id="rId1"/>
+  </tableParts>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0400-000000000000}">
+  <dimension ref="A1:F7"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="1" max="1" width="11.88671875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="18" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="20.44140625" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="22" customWidth="1"/>
+    <col min="5" max="5" width="15" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="11.21875" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A1" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>16</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="E1" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="F1" s="1" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="2" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A2" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="B2" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="C2" s="1">
+        <v>2.3830198725143099E-2</v>
+      </c>
+      <c r="D2" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="E2" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="F2" s="1" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="3" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A3" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="B3" s="1" t="s">
+        <v>22</v>
+      </c>
+      <c r="C3" s="1">
+        <v>9.8940003930462081E-2</v>
+      </c>
+      <c r="D3" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="E3" s="1" t="s">
+        <v>23</v>
+      </c>
+      <c r="F3" s="1" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="4" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A4" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="B4" s="1" t="s">
+        <v>24</v>
+      </c>
+      <c r="C4" s="1">
+        <v>6.6832214140167642E-2</v>
+      </c>
+      <c r="D4" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="E4" s="1" t="s">
+        <v>23</v>
+      </c>
+      <c r="F4" s="1" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="5" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A5" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="B5" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="C5" s="1">
+        <v>8.554868239026639E-2</v>
+      </c>
+      <c r="D5" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="E5" s="1" t="s">
+        <v>23</v>
+      </c>
+      <c r="F5" s="1" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="6" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A6" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="B6" s="1" t="s">
+        <v>22</v>
+      </c>
+      <c r="C6" s="1">
+        <v>2.7019692250728311E-2</v>
+      </c>
+      <c r="D6" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="E6" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="F6" s="1" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="7" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A7" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="B7" s="1" t="s">
+        <v>24</v>
+      </c>
+      <c r="C7" s="1">
+        <v>3.0057600886604991E-2</v>
+      </c>
+      <c r="D7" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="E7" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="F7" s="1" t="s">
+        <v>25</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <tableParts count="1">
+    <tablePart r:id="rId1"/>
+  </tableParts>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0500-000000000000}">
+  <dimension ref="A1:B5"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="1" max="2" width="18.44140625" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A1" s="1" t="s">
+        <v>26</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="2" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A2" s="1" t="s">
+        <v>27</v>
+      </c>
+      <c r="B2" s="1" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="3" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A3" s="1" t="s">
+        <v>29</v>
+      </c>
+      <c r="B3" s="1" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="4" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A4" s="1" t="s">
+        <v>30</v>
+      </c>
+      <c r="B4" s="1" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="5" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A5" s="1" t="s">
+        <v>31</v>
+      </c>
+      <c r="B5" s="1" t="s">
+        <v>32</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <tableParts count="1">
+    <tablePart r:id="rId1"/>
+  </tableParts>
 </worksheet>
 </file>
</xml_diff>